<commit_message>
wip - r&r edits
</commit_message>
<xml_diff>
--- a/output/model_organization.xlsx
+++ b/output/model_organization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjs66\local-r-projects\ladi\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{201E20F8-B871-48D5-8030-231D9DCE9C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A5D264-69F7-4E21-95B2-16C81C508F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23040" yWindow="168" windowWidth="23100" windowHeight="13512" xr2:uid="{5D922D10-131B-499C-AED9-1CB0C72A976E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5D922D10-131B-499C-AED9-1CB0C72A976E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="58">
   <si>
     <t>outcome</t>
   </si>
@@ -189,6 +189,27 @@
   </si>
   <si>
     <t>m3.5</t>
+  </si>
+  <si>
+    <t>sensitivity analyses c</t>
+  </si>
+  <si>
+    <t>interaction with quadratic change</t>
+  </si>
+  <si>
+    <t>sidas</t>
+  </si>
+  <si>
+    <t>m1.4</t>
+  </si>
+  <si>
+    <t>m5.4</t>
+  </si>
+  <si>
+    <t>m6.4</t>
+  </si>
+  <si>
+    <t>m8.4</t>
   </si>
 </sst>
 </file>
@@ -569,10 +590,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9A542CA-3DA0-4A5B-98DA-5495AD9C81C0}">
-  <dimension ref="A1:R13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>39</v>
       </c>
@@ -592,7 +613,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="E2" t="s">
         <v>21</v>
       </c>
@@ -603,7 +624,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -623,7 +644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -661,7 +682,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -693,7 +714,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -725,7 +746,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -739,7 +760,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -753,7 +774,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -767,7 +788,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>13</v>
       </c>
@@ -780,8 +801,11 @@
       <c r="F10" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K10" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>15</v>
       </c>
@@ -794,8 +818,11 @@
       <c r="F11" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -808,8 +835,11 @@
       <c r="F12" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="L12" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>19</v>
       </c>
@@ -821,6 +851,44 @@
       </c>
       <c r="F13" t="s">
         <v>20</v>
+      </c>
+      <c r="K13" t="s">
+        <v>54</v>
+      </c>
+      <c r="L13" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K14" t="s">
+        <v>45</v>
+      </c>
+      <c r="L14" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K15" t="s">
+        <v>55</v>
+      </c>
+      <c r="L15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="K16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="11:12" x14ac:dyDescent="0.3">
+      <c r="K17" t="s">
+        <v>57</v>
+      </c>
+      <c r="L17" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>